<commit_message>
feat: enhance quotation functionality and add asset management
- Added TERM_LABELS for better term handling in quotations.
- Updated quotationPayload to include company name from quotationCompany data.
- Introduced quotationAssets.js for managing stamp assets using IndexedDB.
- Implemented functions to save, load, and clear stamp assets and positions.
- Enhanced quotationExcel.js to dynamically generate terms in Excel export.
- Created quotationImport.js for importing product data from Excel files.
- Improved quotationPdf.js to utilize TERM_LABELS and enhance PDF layout and styling.
- Added taxLookup.js for validating and looking up business information by tax code.
</commit_message>
<xml_diff>
--- a/public/templates/bao-gia-minh-triet.xlsx
+++ b/public/templates/bao-gia-minh-triet.xlsx
@@ -216,7 +216,7 @@
 (VND)</t>
   </si>
   <si>
-    <t>TỔNG CỘNG Đã gồm VAT</t>
+    <t>TỔNG CỘNG ĐÃ GỒM VAT</t>
   </si>
   <si>
     <r>
@@ -275,7 +275,7 @@
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -405,13 +405,45 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1C7A49"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF146C3A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4FAF6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="6">
@@ -492,7 +524,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
@@ -596,6 +628,36 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="2" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1370,25 +1432,25 @@
       <c r="F15" s="3"/>
     </row>
     <row r="16" spans="1:8" s="3" customFormat="1" ht="36" x14ac:dyDescent="0.25">
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="40" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C16" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E16" s="28" t="s">
+      <c r="E16" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="F16" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="G16" s="11" t="s">
+      <c r="G16" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="H16" s="42" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1415,15 +1477,15 @@
       </c>
     </row>
     <row r="18" spans="2:10" s="5" customFormat="1" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="31" t="s">
+      <c r="B18" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="27">
+      <c r="C18" s="46"/>
+      <c r="D18" s="46"/>
+      <c r="E18" s="47"/>
+      <c r="F18" s="46"/>
+      <c r="G18" s="48"/>
+      <c r="H18" s="49">
         <f>SUM(H17:H17)</f>
         <v>1100000</v>
       </c>

</xml_diff>